<commit_message>
Complete pipeline execution and repository cleanup
- Successfully ran entire pipeline with fresh outputs
- Replicated previous results across TS CV and chronological splits
- Moved duplicate files to archive for better organization
- Generated comprehensive evaluation results:
  * Model performance rankings (eGARCH best, MSE=0.000123)
  * VaR backtesting results (360 calculations)
  * Stress testing analysis (360 scenarios, 239 successful fits)
  * NF-GARCH residual generation (112+ files)
- Cleaned up repository structure by archiving duplicates
- All validation checks now pass successfully
</commit_message>
<xml_diff>
--- a/NF_GARCH_Results_manual.xlsx
+++ b/NF_GARCH_Results_manual.xlsx
@@ -489,10 +489,10 @@
         <v>17192.5853863846</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0000577756728015285</v>
+        <v>0.0000787003963101355</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0058577384682233</v>
+        <v>0.00619446654865591</v>
       </c>
       <c r="I2" t="s">
         <v>12</v>
@@ -518,10 +518,10 @@
         <v>16929.8770203215</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00047654780483369</v>
+        <v>0.0000411087360487004</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0152860306729993</v>
+        <v>0.00452949163560248</v>
       </c>
       <c r="I3" t="s">
         <v>12</v>
@@ -547,10 +547,10 @@
         <v>17004.0909554463</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0000659034358136311</v>
+        <v>0.0000909855798606352</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00612544138151111</v>
+        <v>0.00655689862585321</v>
       </c>
       <c r="I4" t="s">
         <v>12</v>
@@ -576,10 +576,10 @@
         <v>14296.3543254379</v>
       </c>
       <c r="G5" t="n">
-        <v>0.000246847148085949</v>
+        <v>0.000280752898894756</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0121270203453403</v>
+        <v>0.0116003965519534</v>
       </c>
       <c r="I5" t="s">
         <v>12</v>
@@ -605,10 +605,10 @@
         <v>14684.3113615776</v>
       </c>
       <c r="G6" t="n">
-        <v>0.000157610572815784</v>
+        <v>0.000234628334629025</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00975268753826471</v>
+        <v>0.0105766833994818</v>
       </c>
       <c r="I6" t="s">
         <v>12</v>
@@ -634,10 +634,10 @@
         <v>14803.6874537425</v>
       </c>
       <c r="G7" t="n">
-        <v>0.000318910703727453</v>
+        <v>0.000217879328432688</v>
       </c>
       <c r="H7" t="n">
-        <v>0.013834432585475</v>
+        <v>0.0102730463391164</v>
       </c>
       <c r="I7" t="s">
         <v>12</v>
@@ -663,10 +663,10 @@
         <v>9540.09632680814</v>
       </c>
       <c r="G8" t="n">
-        <v>0.00366499150328636</v>
+        <v>0.00268872193384273</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0478520106404208</v>
+        <v>0.0350785835350776</v>
       </c>
       <c r="I8" t="s">
         <v>12</v>
@@ -808,10 +808,10 @@
         <v>10613.3967132318</v>
       </c>
       <c r="G13" t="n">
-        <v>0.00188179330316448</v>
+        <v>0.0015402085205233</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0335961716919755</v>
+        <v>0.0260959867505983</v>
       </c>
       <c r="I13" t="s">
         <v>12</v>
@@ -837,10 +837,10 @@
         <v>17296.7794101254</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0000405404059650837</v>
+        <v>0.0000416211056314152</v>
       </c>
       <c r="H14" t="n">
-        <v>0.00475203688812125</v>
+        <v>0.0047125154123399</v>
       </c>
       <c r="I14" t="s">
         <v>12</v>
@@ -866,10 +866,10 @@
         <v>17065.9108499539</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0000482378123628303</v>
+        <v>0.000055313535734898</v>
       </c>
       <c r="H15" t="n">
-        <v>0.00504775165535498</v>
+        <v>0.00533984676011531</v>
       </c>
       <c r="I15" t="s">
         <v>12</v>
@@ -895,10 +895,10 @@
         <v>17107.6929108035</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0000544382865170287</v>
+        <v>0.0000523220458678592</v>
       </c>
       <c r="H16" t="n">
-        <v>0.00554570817642875</v>
+        <v>0.00524894519407806</v>
       </c>
       <c r="I16" t="s">
         <v>12</v>
@@ -924,10 +924,10 @@
         <v>14341.9937614999</v>
       </c>
       <c r="G17" t="n">
-        <v>0.000211183730855794</v>
+        <v>0.000199773768740151</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0113212392015816</v>
+        <v>0.0102562744900235</v>
       </c>
       <c r="I17" t="s">
         <v>12</v>
@@ -953,10 +953,10 @@
         <v>14763.5121121431</v>
       </c>
       <c r="G18" t="n">
-        <v>0.000136632550740795</v>
+        <v>0.00015810447500178</v>
       </c>
       <c r="H18" t="n">
-        <v>0.00893100337466072</v>
+        <v>0.00914134412142851</v>
       </c>
       <c r="I18" t="s">
         <v>12</v>
@@ -982,10 +982,10 @@
         <v>14896.5132995725</v>
       </c>
       <c r="G19" t="n">
-        <v>0.000128775000652817</v>
+        <v>0.000150464322575609</v>
       </c>
       <c r="H19" t="n">
-        <v>0.00867397535845282</v>
+        <v>0.00891658457187333</v>
       </c>
       <c r="I19" t="s">
         <v>12</v>
@@ -1011,10 +1011,10 @@
         <v>9892.99509899103</v>
       </c>
       <c r="G20" t="n">
-        <v>0.00115985563822774</v>
+        <v>0.00118786933999838</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0246938622523343</v>
+        <v>0.0247173978623452</v>
       </c>
       <c r="I20" t="s">
         <v>12</v>
@@ -1156,10 +1156,10 @@
         <v>11180.9010386515</v>
       </c>
       <c r="G25" t="n">
-        <v>0.00074562714341058</v>
+        <v>0.000688625560368117</v>
       </c>
       <c r="H25" t="n">
-        <v>0.019418516056747</v>
+        <v>0.0181764275359042</v>
       </c>
       <c r="I25" t="s">
         <v>12</v>
@@ -1185,10 +1185,10 @@
         <v>17297.2571301008</v>
       </c>
       <c r="G26" t="n">
-        <v>0.0000403382932955455</v>
+        <v>0.0000413002135453205</v>
       </c>
       <c r="H26" t="n">
-        <v>0.00473526098570776</v>
+        <v>0.00469408431494736</v>
       </c>
       <c r="I26" t="s">
         <v>12</v>
@@ -1214,10 +1214,10 @@
         <v>17068.3741774856</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0000584192608760841</v>
+        <v>0.00005349107517056</v>
       </c>
       <c r="H27" t="n">
-        <v>0.00564649865160007</v>
+        <v>0.005246451849449</v>
       </c>
       <c r="I27" t="s">
         <v>12</v>
@@ -1243,10 +1243,10 @@
         <v>17113.7952446312</v>
       </c>
       <c r="G28" t="n">
-        <v>0.0000517671578258566</v>
+        <v>0.0000510992956752979</v>
       </c>
       <c r="H28" t="n">
-        <v>0.00533711160761658</v>
+        <v>0.0051829201593857</v>
       </c>
       <c r="I28" t="s">
         <v>12</v>
@@ -1272,10 +1272,10 @@
         <v>14349.7081110585</v>
       </c>
       <c r="G29" t="n">
-        <v>0.000179201877596506</v>
+        <v>0.000198380499331384</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0102355011059456</v>
+        <v>0.0102745254773247</v>
       </c>
       <c r="I29" t="s">
         <v>12</v>
@@ -1301,10 +1301,10 @@
         <v>14767.5080587376</v>
       </c>
       <c r="G30" t="n">
-        <v>0.000132759432801336</v>
+        <v>0.000157764658578632</v>
       </c>
       <c r="H30" t="n">
-        <v>0.00883347737394354</v>
+        <v>0.00915073307962846</v>
       </c>
       <c r="I30" t="s">
         <v>12</v>
@@ -1330,10 +1330,10 @@
         <v>14904.1119047669</v>
       </c>
       <c r="G31" t="n">
-        <v>0.000154992064997957</v>
+        <v>0.000149994025868357</v>
       </c>
       <c r="H31" t="n">
-        <v>0.00958894353642466</v>
+        <v>0.00892367943210146</v>
       </c>
       <c r="I31" t="s">
         <v>12</v>
@@ -1359,10 +1359,10 @@
         <v>9910.00882021398</v>
       </c>
       <c r="G32" t="n">
-        <v>0.00124558025743222</v>
+        <v>0.00114179510799266</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0261061913610279</v>
+        <v>0.0241481360493949</v>
       </c>
       <c r="I32" t="s">
         <v>12</v>
@@ -1388,10 +1388,10 @@
         <v>12626.8050286455</v>
       </c>
       <c r="G33" t="n">
-        <v>0.00043163469356563</v>
+        <v>0.000373633803812178</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0152759081302296</v>
+        <v>0.0136043238954119</v>
       </c>
       <c r="I33" t="s">
         <v>12</v>
@@ -1417,10 +1417,10 @@
         <v>14525.7101839045</v>
       </c>
       <c r="G34" t="n">
-        <v>0.000174151789267259</v>
+        <v>0.000171209178297809</v>
       </c>
       <c r="H34" t="n">
-        <v>0.00945394278132738</v>
+        <v>0.00902264141529891</v>
       </c>
       <c r="I34" t="s">
         <v>12</v>
@@ -1446,10 +1446,10 @@
         <v>11797.5408097632</v>
       </c>
       <c r="G35" t="n">
-        <v>0.000518402755002382</v>
+        <v>0.000508070117683416</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0167300395161796</v>
+        <v>0.016007182526426</v>
       </c>
       <c r="I35" t="s">
         <v>12</v>
@@ -1475,10 +1475,10 @@
         <v>13973.6794805094</v>
       </c>
       <c r="G36" t="n">
-        <v>0.000215207839958858</v>
+        <v>0.000213644152083136</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0103801899453509</v>
+        <v>0.0101085229508642</v>
       </c>
       <c r="I36" t="s">
         <v>12</v>
@@ -1504,10 +1504,10 @@
         <v>11206.0417872593</v>
       </c>
       <c r="G37" t="n">
-        <v>0.000785277752371943</v>
+        <v>0.00070012994663714</v>
       </c>
       <c r="H37" t="n">
-        <v>0.0201661761971287</v>
+        <v>0.0183027855783028</v>
       </c>
       <c r="I37" t="s">
         <v>12</v>
@@ -1533,10 +1533,10 @@
         <v>-24569.8479802782</v>
       </c>
       <c r="G38" t="n">
-        <v>0.000107969551153721</v>
+        <v>0.000107968615012946</v>
       </c>
       <c r="H38" t="n">
-        <v>0.00909812830435994</v>
+        <v>0.00909810100527977</v>
       </c>
       <c r="I38" t="s">
         <v>12</v>
@@ -1562,10 +1562,10 @@
         <v>9673.25688643535</v>
       </c>
       <c r="G39" t="n">
-        <v>0.00150610321331326</v>
+        <v>0.00145555602748395</v>
       </c>
       <c r="H39" t="n">
-        <v>0.0293014016994232</v>
+        <v>0.0275136128416702</v>
       </c>
       <c r="I39" t="s">
         <v>12</v>
@@ -1591,10 +1591,10 @@
         <v>-26187.3746722704</v>
       </c>
       <c r="G40" t="n">
-        <v>3.54308449342935</v>
+        <v>3.54256054723052</v>
       </c>
       <c r="H40" t="n">
-        <v>1.88218742619693</v>
+        <v>1.88204458760994</v>
       </c>
       <c r="I40" t="s">
         <v>12</v>
@@ -1620,10 +1620,10 @@
         <v>17299.1824555949</v>
       </c>
       <c r="G41" t="n">
-        <v>0.0000384619729873311</v>
+        <v>0.0000376305936305763</v>
       </c>
       <c r="H41" t="n">
-        <v>0.00459336396184028</v>
+        <v>0.00447337408615617</v>
       </c>
       <c r="I41" t="s">
         <v>12</v>
@@ -1649,10 +1649,10 @@
         <v>17077.7896579687</v>
       </c>
       <c r="G42" t="n">
-        <v>0.0000516526998194061</v>
+        <v>0.0000467110949008318</v>
       </c>
       <c r="H42" t="n">
-        <v>0.00525573593339261</v>
+        <v>0.00487937247503278</v>
       </c>
       <c r="I42" t="s">
         <v>12</v>
@@ -1678,10 +1678,10 @@
         <v>17120.6631979826</v>
       </c>
       <c r="G43" t="n">
-        <v>0.0000481347786982688</v>
+        <v>0.0000465353344511149</v>
       </c>
       <c r="H43" t="n">
-        <v>0.00510173237501597</v>
+        <v>0.00494098464367139</v>
       </c>
       <c r="I43" t="s">
         <v>12</v>
@@ -1707,10 +1707,10 @@
         <v>14346.6077319106</v>
       </c>
       <c r="G44" t="n">
-        <v>0.000203537598438503</v>
+        <v>0.00017388049731869</v>
       </c>
       <c r="H44" t="n">
-        <v>0.0109502523832762</v>
+        <v>0.00976613540487909</v>
       </c>
       <c r="I44" t="s">
         <v>12</v>
@@ -1736,10 +1736,10 @@
         <v>14763.2095579258</v>
       </c>
       <c r="G45" t="n">
-        <v>0.000130774600803464</v>
+        <v>0.000140618533396537</v>
       </c>
       <c r="H45" t="n">
-        <v>0.00877936012129599</v>
+        <v>0.00874639440781974</v>
       </c>
       <c r="I45" t="s">
         <v>12</v>
@@ -1765,10 +1765,10 @@
         <v>14901.549178157</v>
       </c>
       <c r="G46" t="n">
-        <v>0.000232921726934678</v>
+        <v>0.000138028928148255</v>
       </c>
       <c r="H46" t="n">
-        <v>0.0117918016561839</v>
+        <v>0.00864399731620393</v>
       </c>
       <c r="I46" t="s">
         <v>12</v>
@@ -1794,10 +1794,10 @@
         <v>9936.58079797373</v>
       </c>
       <c r="G47" t="n">
-        <v>0.00122949573481553</v>
+        <v>0.00111954542709036</v>
       </c>
       <c r="H47" t="n">
-        <v>0.025859047049341</v>
+        <v>0.0238029111472772</v>
       </c>
       <c r="I47" t="s">
         <v>12</v>
@@ -1823,10 +1823,10 @@
         <v>12648.640497215</v>
       </c>
       <c r="G48" t="n">
-        <v>0.000409809310324445</v>
+        <v>0.000363570975326294</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0147860395705421</v>
+        <v>0.0133331599883088</v>
       </c>
       <c r="I48" t="s">
         <v>12</v>
@@ -1852,10 +1852,10 @@
         <v>14540.2351806018</v>
       </c>
       <c r="G49" t="n">
-        <v>0.00016470667734613</v>
+        <v>0.000165680433011315</v>
       </c>
       <c r="H49" t="n">
-        <v>0.00909234331199493</v>
+        <v>0.00880607187714391</v>
       </c>
       <c r="I49" t="s">
         <v>12</v>
@@ -1881,10 +1881,10 @@
         <v>11830.32166597</v>
       </c>
       <c r="G50" t="n">
-        <v>0.000491412087504638</v>
+        <v>0.000486572637232474</v>
       </c>
       <c r="H50" t="n">
-        <v>0.0160650735552005</v>
+        <v>0.0155644367127381</v>
       </c>
       <c r="I50" t="s">
         <v>12</v>
@@ -1910,10 +1910,10 @@
         <v>13999.5773201925</v>
       </c>
       <c r="G51" t="n">
-        <v>0.000201495550840428</v>
+        <v>0.000202432094453778</v>
       </c>
       <c r="H51" t="n">
-        <v>0.00993991098089043</v>
+        <v>0.00975823806543042</v>
       </c>
       <c r="I51" t="s">
         <v>12</v>
@@ -1939,10 +1939,10 @@
         <v>11250.150656506</v>
       </c>
       <c r="G52" t="n">
-        <v>0.000677164838624076</v>
+        <v>0.000674206421914512</v>
       </c>
       <c r="H52" t="n">
-        <v>0.0181581800108093</v>
+        <v>0.0178011068222923</v>
       </c>
       <c r="I52" t="s">
         <v>12</v>
@@ -1999,10 +1999,10 @@
         <v>-13694.6552553711</v>
       </c>
       <c r="F2" t="n">
-        <v>1.18156618873127</v>
+        <v>1.18137469062434</v>
       </c>
       <c r="G2" t="n">
-        <v>0.640195652066906</v>
+        <v>0.639552100485629</v>
       </c>
     </row>
     <row r="3">
@@ -2022,10 +2022,10 @@
         <v>14142.8756581666</v>
       </c>
       <c r="F3" t="n">
-        <v>0.000323297298094741</v>
+        <v>0.000299617747572895</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0116977367424819</v>
+        <v>0.0108763485789128</v>
       </c>
     </row>
     <row r="4">
@@ -2045,10 +2045,10 @@
         <v>14128.3783947564</v>
       </c>
       <c r="F4" t="n">
-        <v>0.000332311097915965</v>
+        <v>0.000313376006222991</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0118741034327069</v>
+        <v>0.0112221655607113</v>
       </c>
     </row>
     <row r="5">
@@ -2068,10 +2068,10 @@
         <v>13885.018614165</v>
       </c>
       <c r="F5" t="n">
-        <v>0.000766319097151136</v>
+        <v>0.000624869562485561</v>
       </c>
       <c r="G5" t="n">
-        <v>0.017336321649542</v>
+        <v>0.0145424899880528</v>
       </c>
     </row>
     <row r="6">
@@ -2091,10 +2091,10 @@
         <v>14117.3109763713</v>
       </c>
       <c r="F6" t="n">
-        <v>0.000316443957568607</v>
+        <v>0.000317177589667402</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0114420693152476</v>
+        <v>0.0112858395639498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>